<commit_message>
Update data files to reflect detailed reporting structure
Refactor data generation scripts and update file metadata to align with a new, standardized data dictionary structure, including specific fields and row counts for each source file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a4d140c7-3570-48e8-a16b-94ef19b602da
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 014fb552-f8d1-4000-bb3f-2379d78dd258
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f90920ee-6a86-4fd5-b8cf-584a7f990b93/a4d140c7-3570-48e8-a16b-94ef19b602da/ST9ErbP
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/public/downloads/MDRM_Taxonomy.xlsx
+++ b/public/downloads/MDRM_Taxonomy.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:L55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,6 +433,9 @@
       <c r="K1" t="str">
         <v>Filing_Requirement</v>
       </c>
+      <c r="L1" t="str">
+        <v>Source_File</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -468,6 +471,9 @@
       <c r="K2" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L2" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -503,6 +509,9 @@
       <c r="K3" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L3" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -538,6 +547,9 @@
       <c r="K4" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L4" t="str">
+        <v>Loan_Portfolio</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -573,6 +585,9 @@
       <c r="K5" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L5" t="str">
+        <v>Treasury_Data</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -608,6 +623,9 @@
       <c r="K6" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L6" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -643,6 +661,9 @@
       <c r="K7" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L7" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -678,6 +699,9 @@
       <c r="K8" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L8" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -713,6 +737,9 @@
       <c r="K9" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L9" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -748,6 +775,9 @@
       <c r="K10" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L10" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -783,6 +813,9 @@
       <c r="K11" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L11" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -818,6 +851,9 @@
       <c r="K12" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L12" t="str">
+        <v>GL_Extract</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -853,6 +889,9 @@
       <c r="K13" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L13" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -888,6 +927,9 @@
       <c r="K14" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L14" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -923,6 +965,9 @@
       <c r="K15" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L15" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -958,6 +1003,9 @@
       <c r="K16" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L16" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -993,6 +1041,9 @@
       <c r="K17" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L17" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1028,6 +1079,9 @@
       <c r="K18" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L18" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1063,60 +1117,66 @@
       <c r="K19" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L19" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>UBPR1</v>
+        <v>RCFDC223</v>
       </c>
       <c r="B20" t="str">
-        <v>Net Interest Margin</v>
+        <v>Leverage Ratio</v>
       </c>
       <c r="C20" t="str">
-        <v>UBPR Page 1</v>
+        <v>RC-R Part I</v>
       </c>
       <c r="D20" t="str">
-        <v>Line 4</v>
+        <v>Line 35</v>
       </c>
       <c r="E20" t="str">
-        <v>Performance Ratios</v>
+        <v>Capital Ratios</v>
       </c>
       <c r="F20" t="str">
-        <v>Net interest income / average earning assets annualized</v>
+        <v>Tier 1 capital / average total consolidated assets</v>
       </c>
       <c r="G20" t="str">
         <v>Percent</v>
       </c>
       <c r="H20" t="str">
-        <v>UBPR</v>
+        <v>RCFD</v>
       </c>
       <c r="I20" t="str">
-        <v>NIMY</v>
+        <v>C223</v>
       </c>
       <c r="J20" t="str">
-        <v>UBPR</v>
+        <v>Basel III</v>
       </c>
       <c r="K20" t="str">
-        <v>Derived</v>
+        <v>Mandatory</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Risk_Metrics</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>UBPR2</v>
+        <v>UBPR1</v>
       </c>
       <c r="B21" t="str">
-        <v>Return on Assets</v>
+        <v>Net Interest Margin</v>
       </c>
       <c r="C21" t="str">
         <v>UBPR Page 1</v>
       </c>
       <c r="D21" t="str">
-        <v>Line 1</v>
+        <v>Line 4</v>
       </c>
       <c r="E21" t="str">
         <v>Performance Ratios</v>
       </c>
       <c r="F21" t="str">
-        <v>Net income / average total assets annualized</v>
+        <v>Net interest income / average earning assets annualized</v>
       </c>
       <c r="G21" t="str">
         <v>Percent</v>
@@ -1125,7 +1185,7 @@
         <v>UBPR</v>
       </c>
       <c r="I21" t="str">
-        <v>ROA</v>
+        <v>NIMY</v>
       </c>
       <c r="J21" t="str">
         <v>UBPR</v>
@@ -1133,25 +1193,28 @@
       <c r="K21" t="str">
         <v>Derived</v>
       </c>
+      <c r="L21" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>UBPR3</v>
+        <v>UBPR2</v>
       </c>
       <c r="B22" t="str">
-        <v>Return on Equity</v>
+        <v>Return on Assets</v>
       </c>
       <c r="C22" t="str">
         <v>UBPR Page 1</v>
       </c>
       <c r="D22" t="str">
-        <v>Line 2</v>
+        <v>Line 1</v>
       </c>
       <c r="E22" t="str">
         <v>Performance Ratios</v>
       </c>
       <c r="F22" t="str">
-        <v>Net income / average equity annualized</v>
+        <v>Net income / average total assets annualized</v>
       </c>
       <c r="G22" t="str">
         <v>Percent</v>
@@ -1160,7 +1223,7 @@
         <v>UBPR</v>
       </c>
       <c r="I22" t="str">
-        <v>ROE</v>
+        <v>ROA</v>
       </c>
       <c r="J22" t="str">
         <v>UBPR</v>
@@ -1168,25 +1231,28 @@
       <c r="K22" t="str">
         <v>Derived</v>
       </c>
+      <c r="L22" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>UBPR4</v>
+        <v>UBPR3</v>
       </c>
       <c r="B23" t="str">
-        <v>Efficiency Ratio</v>
+        <v>Return on Equity</v>
       </c>
       <c r="C23" t="str">
         <v>UBPR Page 1</v>
       </c>
       <c r="D23" t="str">
-        <v>Line 8</v>
+        <v>Line 2</v>
       </c>
       <c r="E23" t="str">
         <v>Performance Ratios</v>
       </c>
       <c r="F23" t="str">
-        <v>Non-interest expense / (net interest income + non-interest income)</v>
+        <v>Net income / average equity annualized</v>
       </c>
       <c r="G23" t="str">
         <v>Percent</v>
@@ -1195,7 +1261,7 @@
         <v>UBPR</v>
       </c>
       <c r="I23" t="str">
-        <v>EEFF</v>
+        <v>ROE</v>
       </c>
       <c r="J23" t="str">
         <v>UBPR</v>
@@ -1203,25 +1269,28 @@
       <c r="K23" t="str">
         <v>Derived</v>
       </c>
+      <c r="L23" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>UBPR5</v>
+        <v>UBPR4</v>
       </c>
       <c r="B24" t="str">
-        <v>NPA Ratio</v>
+        <v>Efficiency Ratio</v>
       </c>
       <c r="C24" t="str">
-        <v>UBPR Page 7</v>
+        <v>UBPR Page 1</v>
       </c>
       <c r="D24" t="str">
-        <v>Line 15</v>
+        <v>Line 8</v>
       </c>
       <c r="E24" t="str">
-        <v>Asset Quality</v>
+        <v>Performance Ratios</v>
       </c>
       <c r="F24" t="str">
-        <v>Non-performing assets / total assets</v>
+        <v>Non-interest expense / (net interest income + non-interest income)</v>
       </c>
       <c r="G24" t="str">
         <v>Percent</v>
@@ -1230,7 +1299,7 @@
         <v>UBPR</v>
       </c>
       <c r="I24" t="str">
-        <v>P3ASSET</v>
+        <v>EEFF</v>
       </c>
       <c r="J24" t="str">
         <v>UBPR</v>
@@ -1238,25 +1307,28 @@
       <c r="K24" t="str">
         <v>Derived</v>
       </c>
+      <c r="L24" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>UBPR6</v>
+        <v>UBPR5</v>
       </c>
       <c r="B25" t="str">
-        <v>Net Charge-Off Rate</v>
+        <v>NPA Ratio</v>
       </c>
       <c r="C25" t="str">
-        <v>UBPR Page 4</v>
+        <v>UBPR Page 7</v>
       </c>
       <c r="D25" t="str">
-        <v>Line 6</v>
+        <v>Line 15</v>
       </c>
       <c r="E25" t="str">
         <v>Asset Quality</v>
       </c>
       <c r="F25" t="str">
-        <v>Net charge-offs / average loans annualized</v>
+        <v>Non-performing assets / total assets</v>
       </c>
       <c r="G25" t="str">
         <v>Percent</v>
@@ -1265,7 +1337,7 @@
         <v>UBPR</v>
       </c>
       <c r="I25" t="str">
-        <v>ELNANTR</v>
+        <v>P3ASSET</v>
       </c>
       <c r="J25" t="str">
         <v>UBPR</v>
@@ -1273,25 +1345,28 @@
       <c r="K25" t="str">
         <v>Derived</v>
       </c>
+      <c r="L25" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>UBPR7</v>
+        <v>UBPR6</v>
       </c>
       <c r="B26" t="str">
-        <v>Loan to Deposit Ratio</v>
+        <v>Net Charge-Off Rate</v>
       </c>
       <c r="C26" t="str">
-        <v>UBPR Page 1</v>
+        <v>UBPR Page 4</v>
       </c>
       <c r="D26" t="str">
-        <v>Line 12</v>
+        <v>Line 6</v>
       </c>
       <c r="E26" t="str">
-        <v>Liquidity</v>
+        <v>Asset Quality</v>
       </c>
       <c r="F26" t="str">
-        <v>Total loans / total deposits</v>
+        <v>Net charge-offs / average loans annualized</v>
       </c>
       <c r="G26" t="str">
         <v>Percent</v>
@@ -1300,7 +1375,7 @@
         <v>UBPR</v>
       </c>
       <c r="I26" t="str">
-        <v>LDEP</v>
+        <v>ELNANTR</v>
       </c>
       <c r="J26" t="str">
         <v>UBPR</v>
@@ -1308,60 +1383,66 @@
       <c r="K26" t="str">
         <v>Derived</v>
       </c>
+      <c r="L26" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>RCON6631</v>
+        <v>UBPR7</v>
       </c>
       <c r="B27" t="str">
-        <v>Deposits - Demand (Non-Interest)</v>
+        <v>Loan to Deposit Ratio</v>
       </c>
       <c r="C27" t="str">
-        <v>RC-E Part I</v>
+        <v>UBPR Page 1</v>
       </c>
       <c r="D27" t="str">
-        <v>Line 1</v>
+        <v>Line 12</v>
       </c>
       <c r="E27" t="str">
-        <v>Deposits</v>
+        <v>Liquidity</v>
       </c>
       <c r="F27" t="str">
-        <v>Non-interest bearing demand deposits (domestic)</v>
+        <v>Total loans / total deposits</v>
       </c>
       <c r="G27" t="str">
-        <v>Thousands USD</v>
+        <v>Percent</v>
       </c>
       <c r="H27" t="str">
-        <v>RCON</v>
+        <v>UBPR</v>
       </c>
       <c r="I27" t="str">
-        <v>6631</v>
+        <v>LDEP</v>
       </c>
       <c r="J27" t="str">
-        <v>N/A</v>
+        <v>UBPR</v>
       </c>
       <c r="K27" t="str">
-        <v>Mandatory</v>
+        <v>Derived</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Risk_Metrics</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>RCON6636</v>
+        <v>RCON6631</v>
       </c>
       <c r="B28" t="str">
-        <v>Deposits - NOW Accounts</v>
+        <v>Deposits - Demand (Non-Interest)</v>
       </c>
       <c r="C28" t="str">
         <v>RC-E Part I</v>
       </c>
       <c r="D28" t="str">
-        <v>Line 2</v>
+        <v>Line 1</v>
       </c>
       <c r="E28" t="str">
         <v>Deposits</v>
       </c>
       <c r="F28" t="str">
-        <v>Interest-bearing transaction accounts</v>
+        <v>Non-interest bearing demand deposits (domestic)</v>
       </c>
       <c r="G28" t="str">
         <v>Thousands USD</v>
@@ -1370,33 +1451,36 @@
         <v>RCON</v>
       </c>
       <c r="I28" t="str">
-        <v>6636</v>
+        <v>6631</v>
       </c>
       <c r="J28" t="str">
         <v>N/A</v>
       </c>
       <c r="K28" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L28" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>RCON2389</v>
+        <v>RCON6636</v>
       </c>
       <c r="B29" t="str">
-        <v>Deposits - MMDA</v>
+        <v>Deposits - NOW Accounts</v>
       </c>
       <c r="C29" t="str">
         <v>RC-E Part I</v>
       </c>
       <c r="D29" t="str">
-        <v>Line 3</v>
+        <v>Line 2</v>
       </c>
       <c r="E29" t="str">
         <v>Deposits</v>
       </c>
       <c r="F29" t="str">
-        <v>Money market deposit accounts</v>
+        <v>Interest-bearing transaction accounts</v>
       </c>
       <c r="G29" t="str">
         <v>Thousands USD</v>
@@ -1405,33 +1489,36 @@
         <v>RCON</v>
       </c>
       <c r="I29" t="str">
-        <v>2389</v>
+        <v>6636</v>
       </c>
       <c r="J29" t="str">
         <v>N/A</v>
       </c>
       <c r="K29" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L29" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>RCON6648</v>
+        <v>RCON2389</v>
       </c>
       <c r="B30" t="str">
-        <v>Deposits - Other Savings</v>
+        <v>Deposits - MMDA</v>
       </c>
       <c r="C30" t="str">
         <v>RC-E Part I</v>
       </c>
       <c r="D30" t="str">
-        <v>Line 4</v>
+        <v>Line 3</v>
       </c>
       <c r="E30" t="str">
         <v>Deposits</v>
       </c>
       <c r="F30" t="str">
-        <v>Other savings deposits</v>
+        <v>Money market deposit accounts</v>
       </c>
       <c r="G30" t="str">
         <v>Thousands USD</v>
@@ -1440,33 +1527,36 @@
         <v>RCON</v>
       </c>
       <c r="I30" t="str">
-        <v>6648</v>
+        <v>2389</v>
       </c>
       <c r="J30" t="str">
         <v>N/A</v>
       </c>
       <c r="K30" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L30" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>RCON6645</v>
+        <v>RCON6648</v>
       </c>
       <c r="B31" t="str">
-        <v>Deposits - Time &lt; $250K</v>
+        <v>Deposits - Other Savings</v>
       </c>
       <c r="C31" t="str">
         <v>RC-E Part I</v>
       </c>
       <c r="D31" t="str">
-        <v>Line 5</v>
+        <v>Line 4</v>
       </c>
       <c r="E31" t="str">
         <v>Deposits</v>
       </c>
       <c r="F31" t="str">
-        <v>Time deposits less than $250,000</v>
+        <v>Other savings deposits</v>
       </c>
       <c r="G31" t="str">
         <v>Thousands USD</v>
@@ -1475,33 +1565,36 @@
         <v>RCON</v>
       </c>
       <c r="I31" t="str">
-        <v>6645</v>
+        <v>6648</v>
       </c>
       <c r="J31" t="str">
         <v>N/A</v>
       </c>
       <c r="K31" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L31" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>RCONJ473</v>
+        <v>RCON6645</v>
       </c>
       <c r="B32" t="str">
-        <v>Deposits - Time &gt;= $250K</v>
+        <v>Deposits - Time &lt; $250K</v>
       </c>
       <c r="C32" t="str">
         <v>RC-E Part I</v>
       </c>
       <c r="D32" t="str">
-        <v>Line 6</v>
+        <v>Line 5</v>
       </c>
       <c r="E32" t="str">
         <v>Deposits</v>
       </c>
       <c r="F32" t="str">
-        <v>Time deposits $250,000 or more</v>
+        <v>Time deposits less than $250,000</v>
       </c>
       <c r="G32" t="str">
         <v>Thousands USD</v>
@@ -1510,68 +1603,74 @@
         <v>RCON</v>
       </c>
       <c r="I32" t="str">
-        <v>J473</v>
+        <v>6645</v>
       </c>
       <c r="J32" t="str">
         <v>N/A</v>
       </c>
       <c r="K32" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L32" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>RCFD1754</v>
+        <v>RCONJ473</v>
       </c>
       <c r="B33" t="str">
-        <v>Loans - C&amp;I (Domestic)</v>
+        <v>Deposits - Time &gt;= $250K</v>
       </c>
       <c r="C33" t="str">
-        <v>RC-C Part I</v>
+        <v>RC-E Part I</v>
       </c>
       <c r="D33" t="str">
-        <v>Line 4.a</v>
+        <v>Line 6</v>
       </c>
       <c r="E33" t="str">
-        <v>Loans</v>
+        <v>Deposits</v>
       </c>
       <c r="F33" t="str">
-        <v>Commercial and industrial loans to US addresses</v>
+        <v>Time deposits $250,000 or more</v>
       </c>
       <c r="G33" t="str">
         <v>Thousands USD</v>
       </c>
       <c r="H33" t="str">
-        <v>RCFD</v>
+        <v>RCON</v>
       </c>
       <c r="I33" t="str">
-        <v>1754</v>
+        <v>J473</v>
       </c>
       <c r="J33" t="str">
         <v>N/A</v>
       </c>
       <c r="K33" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L33" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>RCFD1763</v>
+        <v>RCFD1754</v>
       </c>
       <c r="B34" t="str">
-        <v>Loans - CRE (Non-Farm, Non-Res)</v>
+        <v>Loans - C&amp;I (Domestic)</v>
       </c>
       <c r="C34" t="str">
         <v>RC-C Part I</v>
       </c>
       <c r="D34" t="str">
-        <v>Line 1.a.(1)</v>
+        <v>Line 4.a</v>
       </c>
       <c r="E34" t="str">
         <v>Loans</v>
       </c>
       <c r="F34" t="str">
-        <v>Non-farm non-residential CRE loans</v>
+        <v>Commercial and industrial loans to US addresses</v>
       </c>
       <c r="G34" t="str">
         <v>Thousands USD</v>
@@ -1580,33 +1679,36 @@
         <v>RCFD</v>
       </c>
       <c r="I34" t="str">
-        <v>1763</v>
+        <v>1754</v>
       </c>
       <c r="J34" t="str">
         <v>N/A</v>
       </c>
       <c r="K34" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>RCFD1764</v>
+        <v>RCFD1763</v>
       </c>
       <c r="B35" t="str">
-        <v>Loans - CRE (Multifamily)</v>
+        <v>Loans - CRE (Non-Farm, Non-Res)</v>
       </c>
       <c r="C35" t="str">
         <v>RC-C Part I</v>
       </c>
       <c r="D35" t="str">
-        <v>Line 1.a.(2)</v>
+        <v>Line 1.a.(1)</v>
       </c>
       <c r="E35" t="str">
         <v>Loans</v>
       </c>
       <c r="F35" t="str">
-        <v>Multifamily residential real estate loans</v>
+        <v>Non-farm non-residential CRE loans</v>
       </c>
       <c r="G35" t="str">
         <v>Thousands USD</v>
@@ -1615,33 +1717,36 @@
         <v>RCFD</v>
       </c>
       <c r="I35" t="str">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="J35" t="str">
         <v>N/A</v>
       </c>
       <c r="K35" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>RCFD1460</v>
+        <v>RCFD1764</v>
       </c>
       <c r="B36" t="str">
-        <v>Loans - Construction &amp; Land</v>
+        <v>Loans - CRE (Multifamily)</v>
       </c>
       <c r="C36" t="str">
         <v>RC-C Part I</v>
       </c>
       <c r="D36" t="str">
-        <v>Line 1.a.(3)</v>
+        <v>Line 1.a.(2)</v>
       </c>
       <c r="E36" t="str">
         <v>Loans</v>
       </c>
       <c r="F36" t="str">
-        <v>Construction and land development loans</v>
+        <v>Multifamily residential real estate loans</v>
       </c>
       <c r="G36" t="str">
         <v>Thousands USD</v>
@@ -1650,33 +1755,36 @@
         <v>RCFD</v>
       </c>
       <c r="I36" t="str">
-        <v>1460</v>
+        <v>1764</v>
       </c>
       <c r="J36" t="str">
         <v>N/A</v>
       </c>
       <c r="K36" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>RCFD1797</v>
+        <v>RCFD1460</v>
       </c>
       <c r="B37" t="str">
-        <v>Loans - 1-4 Family Residential</v>
+        <v>Loans - Construction &amp; Land</v>
       </c>
       <c r="C37" t="str">
         <v>RC-C Part I</v>
       </c>
       <c r="D37" t="str">
-        <v>Line 1.c</v>
+        <v>Line 1.a.(3)</v>
       </c>
       <c r="E37" t="str">
         <v>Loans</v>
       </c>
       <c r="F37" t="str">
-        <v>Residential real estate loans 1-4 family</v>
+        <v>Construction and land development loans</v>
       </c>
       <c r="G37" t="str">
         <v>Thousands USD</v>
@@ -1685,33 +1793,36 @@
         <v>RCFD</v>
       </c>
       <c r="I37" t="str">
-        <v>1797</v>
+        <v>1460</v>
       </c>
       <c r="J37" t="str">
         <v>N/A</v>
       </c>
       <c r="K37" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>RCFD2107</v>
+        <v>RCFD1797</v>
       </c>
       <c r="B38" t="str">
-        <v>Allowance for Credit Losses</v>
+        <v>Loans - 1-4 Family Residential</v>
       </c>
       <c r="C38" t="str">
-        <v>RC</v>
+        <v>RC-C Part I</v>
       </c>
       <c r="D38" t="str">
-        <v>Line 4.c</v>
+        <v>Line 1.c</v>
       </c>
       <c r="E38" t="str">
         <v>Loans</v>
       </c>
       <c r="F38" t="str">
-        <v>Total allowance for credit losses on loans</v>
+        <v>Residential real estate loans 1-4 family</v>
       </c>
       <c r="G38" t="str">
         <v>Thousands USD</v>
@@ -1720,33 +1831,36 @@
         <v>RCFD</v>
       </c>
       <c r="I38" t="str">
-        <v>2107</v>
+        <v>1797</v>
       </c>
       <c r="J38" t="str">
-        <v>ASC 326</v>
+        <v>N/A</v>
       </c>
       <c r="K38" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>RCFDB528</v>
+        <v>RCFD2107</v>
       </c>
       <c r="B39" t="str">
-        <v>HTM Securities - Amortized Cost</v>
+        <v>Allowance for Credit Losses</v>
       </c>
       <c r="C39" t="str">
-        <v>RC-B</v>
+        <v>RC</v>
       </c>
       <c r="D39" t="str">
-        <v>Line 8.a</v>
+        <v>Line 4.c</v>
       </c>
       <c r="E39" t="str">
-        <v>Securities</v>
+        <v>Loans</v>
       </c>
       <c r="F39" t="str">
-        <v>Held-to-maturity debt securities at amortized cost</v>
+        <v>Total allowance for credit losses on loans</v>
       </c>
       <c r="G39" t="str">
         <v>Thousands USD</v>
@@ -1755,33 +1869,36 @@
         <v>RCFD</v>
       </c>
       <c r="I39" t="str">
-        <v>B528</v>
+        <v>2107</v>
       </c>
       <c r="J39" t="str">
-        <v>ASC 320</v>
+        <v>ASC 326</v>
       </c>
       <c r="K39" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Loan_Portfolio</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>RCFDB529</v>
+        <v>RCFDB528</v>
       </c>
       <c r="B40" t="str">
-        <v>HTM Securities - Fair Value</v>
+        <v>HTM Securities - Amortized Cost</v>
       </c>
       <c r="C40" t="str">
         <v>RC-B</v>
       </c>
       <c r="D40" t="str">
-        <v>Line 8.b</v>
+        <v>Line 8.a</v>
       </c>
       <c r="E40" t="str">
         <v>Securities</v>
       </c>
       <c r="F40" t="str">
-        <v>Held-to-maturity debt securities at fair value</v>
+        <v>Held-to-maturity debt securities at amortized cost</v>
       </c>
       <c r="G40" t="str">
         <v>Thousands USD</v>
@@ -1790,7 +1907,7 @@
         <v>RCFD</v>
       </c>
       <c r="I40" t="str">
-        <v>B529</v>
+        <v>B528</v>
       </c>
       <c r="J40" t="str">
         <v>ASC 320</v>
@@ -1798,25 +1915,28 @@
       <c r="K40" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L40" t="str">
+        <v>Treasury_Data</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>RCFD1773</v>
+        <v>RCFDB529</v>
       </c>
       <c r="B41" t="str">
-        <v>AFS Securities - Fair Value</v>
+        <v>HTM Securities - Fair Value</v>
       </c>
       <c r="C41" t="str">
         <v>RC-B</v>
       </c>
       <c r="D41" t="str">
-        <v>Line 8.c</v>
+        <v>Line 8.b</v>
       </c>
       <c r="E41" t="str">
         <v>Securities</v>
       </c>
       <c r="F41" t="str">
-        <v>Available-for-sale debt securities at fair value</v>
+        <v>Held-to-maturity debt securities at fair value</v>
       </c>
       <c r="G41" t="str">
         <v>Thousands USD</v>
@@ -1825,7 +1945,7 @@
         <v>RCFD</v>
       </c>
       <c r="I41" t="str">
-        <v>1773</v>
+        <v>B529</v>
       </c>
       <c r="J41" t="str">
         <v>ASC 320</v>
@@ -1833,25 +1953,28 @@
       <c r="K41" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L41" t="str">
+        <v>Treasury_Data</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>RCFDB530</v>
+        <v>RCFD1773</v>
       </c>
       <c r="B42" t="str">
-        <v>AFS Securities - Amortized Cost</v>
+        <v>AFS Securities - Fair Value</v>
       </c>
       <c r="C42" t="str">
         <v>RC-B</v>
       </c>
       <c r="D42" t="str">
-        <v>Line 8.d</v>
+        <v>Line 8.c</v>
       </c>
       <c r="E42" t="str">
         <v>Securities</v>
       </c>
       <c r="F42" t="str">
-        <v>Available-for-sale debt securities amortized cost</v>
+        <v>Available-for-sale debt securities at fair value</v>
       </c>
       <c r="G42" t="str">
         <v>Thousands USD</v>
@@ -1860,7 +1983,7 @@
         <v>RCFD</v>
       </c>
       <c r="I42" t="str">
-        <v>B530</v>
+        <v>1773</v>
       </c>
       <c r="J42" t="str">
         <v>ASC 320</v>
@@ -1868,25 +1991,28 @@
       <c r="K42" t="str">
         <v>Mandatory</v>
       </c>
+      <c r="L42" t="str">
+        <v>Treasury_Data</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>RCFDC026</v>
+        <v>RCFDB530</v>
       </c>
       <c r="B43" t="str">
-        <v>AOCI - Unrealized G/L on AFS</v>
+        <v>AFS Securities - Amortized Cost</v>
       </c>
       <c r="C43" t="str">
-        <v>RC-R Part I</v>
+        <v>RC-B</v>
       </c>
       <c r="D43" t="str">
-        <v>Line 3.a</v>
+        <v>Line 8.d</v>
       </c>
       <c r="E43" t="str">
-        <v>Capital</v>
+        <v>Securities</v>
       </c>
       <c r="F43" t="str">
-        <v>Accumulated other comprehensive income - AFS securities</v>
+        <v>Available-for-sale debt securities amortized cost</v>
       </c>
       <c r="G43" t="str">
         <v>Thousands USD</v>
@@ -1895,68 +2021,74 @@
         <v>RCFD</v>
       </c>
       <c r="I43" t="str">
-        <v>C026</v>
+        <v>B530</v>
       </c>
       <c r="J43" t="str">
-        <v>ASC 220</v>
+        <v>ASC 320</v>
       </c>
       <c r="K43" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Treasury_Data</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>RIAD4010</v>
+        <v>RCFDC026</v>
       </c>
       <c r="B44" t="str">
-        <v>Interest on Loans</v>
+        <v>AOCI - Unrealized G/L on AFS</v>
       </c>
       <c r="C44" t="str">
-        <v>RI</v>
+        <v>RC-R Part I</v>
       </c>
       <c r="D44" t="str">
-        <v>Line 1.a</v>
+        <v>Line 3.a</v>
       </c>
       <c r="E44" t="str">
-        <v>Interest Income</v>
+        <v>Capital</v>
       </c>
       <c r="F44" t="str">
-        <v>Interest and fee income on loans</v>
+        <v>Accumulated other comprehensive income - AFS securities</v>
       </c>
       <c r="G44" t="str">
         <v>Thousands USD</v>
       </c>
       <c r="H44" t="str">
-        <v>RIAD</v>
+        <v>RCFD</v>
       </c>
       <c r="I44" t="str">
-        <v>4010</v>
+        <v>C026</v>
       </c>
       <c r="J44" t="str">
-        <v>N/A</v>
+        <v>ASC 220</v>
       </c>
       <c r="K44" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L44" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>RIAD4020</v>
+        <v>RIAD4010</v>
       </c>
       <c r="B45" t="str">
-        <v>Interest on Investment Securities</v>
+        <v>Interest on Loans</v>
       </c>
       <c r="C45" t="str">
         <v>RI</v>
       </c>
       <c r="D45" t="str">
-        <v>Line 1.b</v>
+        <v>Line 1.a</v>
       </c>
       <c r="E45" t="str">
         <v>Interest Income</v>
       </c>
       <c r="F45" t="str">
-        <v>Interest income on held-to-maturity securities</v>
+        <v>Interest and fee income on loans</v>
       </c>
       <c r="G45" t="str">
         <v>Thousands USD</v>
@@ -1965,33 +2097,36 @@
         <v>RIAD</v>
       </c>
       <c r="I45" t="str">
-        <v>4020</v>
+        <v>4010</v>
       </c>
       <c r="J45" t="str">
         <v>N/A</v>
       </c>
       <c r="K45" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L45" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>RIAD4115</v>
+        <v>RIAD4020</v>
       </c>
       <c r="B46" t="str">
-        <v>Interest on Deposits</v>
+        <v>Interest on Investment Securities</v>
       </c>
       <c r="C46" t="str">
         <v>RI</v>
       </c>
       <c r="D46" t="str">
-        <v>Line 2.a</v>
+        <v>Line 1.b</v>
       </c>
       <c r="E46" t="str">
-        <v>Interest Expense</v>
+        <v>Interest Income</v>
       </c>
       <c r="F46" t="str">
-        <v>Interest expense on deposits</v>
+        <v>Interest income on held-to-maturity securities</v>
       </c>
       <c r="G46" t="str">
         <v>Thousands USD</v>
@@ -2000,33 +2135,36 @@
         <v>RIAD</v>
       </c>
       <c r="I46" t="str">
-        <v>4115</v>
+        <v>4020</v>
       </c>
       <c r="J46" t="str">
         <v>N/A</v>
       </c>
       <c r="K46" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L46" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>RIAD4180</v>
+        <v>RIAD4115</v>
       </c>
       <c r="B47" t="str">
-        <v>Salaries and Employee Benefits</v>
+        <v>Interest on Deposits</v>
       </c>
       <c r="C47" t="str">
         <v>RI</v>
       </c>
       <c r="D47" t="str">
-        <v>Line 7.a</v>
+        <v>Line 2.a</v>
       </c>
       <c r="E47" t="str">
-        <v>Non-Interest Expense</v>
+        <v>Interest Expense</v>
       </c>
       <c r="F47" t="str">
-        <v>Total salaries and employee benefits</v>
+        <v>Interest expense on deposits</v>
       </c>
       <c r="G47" t="str">
         <v>Thousands USD</v>
@@ -2035,33 +2173,36 @@
         <v>RIAD</v>
       </c>
       <c r="I47" t="str">
-        <v>4180</v>
+        <v>4115</v>
       </c>
       <c r="J47" t="str">
         <v>N/A</v>
       </c>
       <c r="K47" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L47" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RIADA220</v>
+        <v>RIAD4180</v>
       </c>
       <c r="B48" t="str">
-        <v>Trading Revenue</v>
+        <v>Salaries and Employee Benefits</v>
       </c>
       <c r="C48" t="str">
         <v>RI</v>
       </c>
       <c r="D48" t="str">
-        <v>Line 5.c</v>
+        <v>Line 7.a</v>
       </c>
       <c r="E48" t="str">
-        <v>Non-Interest Income</v>
+        <v>Non-Interest Expense</v>
       </c>
       <c r="F48" t="str">
-        <v>Trading revenue from all asset classes</v>
+        <v>Total salaries and employee benefits</v>
       </c>
       <c r="G48" t="str">
         <v>Thousands USD</v>
@@ -2070,33 +2211,36 @@
         <v>RIAD</v>
       </c>
       <c r="I48" t="str">
-        <v>A220</v>
+        <v>4180</v>
       </c>
       <c r="J48" t="str">
         <v>N/A</v>
       </c>
       <c r="K48" t="str">
-        <v>Conditional</v>
+        <v>Mandatory</v>
+      </c>
+      <c r="L48" t="str">
+        <v>GL_Extract</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RIAD3196</v>
+        <v>RIADA220</v>
       </c>
       <c r="B49" t="str">
-        <v>Realized G/L on Securities</v>
+        <v>Trading Revenue</v>
       </c>
       <c r="C49" t="str">
         <v>RI</v>
       </c>
       <c r="D49" t="str">
-        <v>Line 6.a</v>
+        <v>Line 5.c</v>
       </c>
       <c r="E49" t="str">
         <v>Non-Interest Income</v>
       </c>
       <c r="F49" t="str">
-        <v>Realized gains (losses) on HTM and AFS securities</v>
+        <v>Trading revenue from all asset classes</v>
       </c>
       <c r="G49" t="str">
         <v>Thousands USD</v>
@@ -2105,103 +2249,112 @@
         <v>RIAD</v>
       </c>
       <c r="I49" t="str">
-        <v>3196</v>
+        <v>A220</v>
       </c>
       <c r="J49" t="str">
-        <v>ASC 320</v>
+        <v>N/A</v>
       </c>
       <c r="K49" t="str">
-        <v>Mandatory</v>
+        <v>Conditional</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Trading_Positions</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RCFDC223</v>
+        <v>RIAD3196</v>
       </c>
       <c r="B50" t="str">
-        <v>Leverage Ratio</v>
+        <v>Realized G/L on Securities</v>
       </c>
       <c r="C50" t="str">
-        <v>RC-R Part I</v>
+        <v>RI</v>
       </c>
       <c r="D50" t="str">
-        <v>Line 35</v>
+        <v>Line 6.a</v>
       </c>
       <c r="E50" t="str">
-        <v>Capital Ratios</v>
+        <v>Non-Interest Income</v>
       </c>
       <c r="F50" t="str">
-        <v>Tier 1 capital / average total consolidated assets</v>
+        <v>Realized gains (losses) on HTM and AFS securities</v>
       </c>
       <c r="G50" t="str">
-        <v>Percent</v>
+        <v>Thousands USD</v>
       </c>
       <c r="H50" t="str">
-        <v>RCFD</v>
+        <v>RIAD</v>
       </c>
       <c r="I50" t="str">
-        <v>C223</v>
+        <v>3196</v>
       </c>
       <c r="J50" t="str">
-        <v>Basel III</v>
+        <v>ASC 320</v>
       </c>
       <c r="K50" t="str">
         <v>Mandatory</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Treasury_Data</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>BHCK4340</v>
+        <v>RCON3545</v>
       </c>
       <c r="B51" t="str">
-        <v>BHC Net Income</v>
+        <v>Trading Assets</v>
       </c>
       <c r="C51" t="str">
-        <v>FR Y-9C</v>
+        <v>RC</v>
       </c>
       <c r="D51" t="str">
-        <v>HC-Line 14</v>
+        <v>Line 5</v>
       </c>
       <c r="E51" t="str">
-        <v>BHC Income</v>
+        <v>Balance Sheet</v>
       </c>
       <c r="F51" t="str">
-        <v>Consolidated net income for bank holding company</v>
+        <v>Total trading assets at fair value</v>
       </c>
       <c r="G51" t="str">
         <v>Thousands USD</v>
       </c>
       <c r="H51" t="str">
-        <v>BHCK</v>
+        <v>RCON</v>
       </c>
       <c r="I51" t="str">
-        <v>4340</v>
+        <v>3545</v>
       </c>
       <c r="J51" t="str">
-        <v>FR Y-9C</v>
+        <v>ASC 820</v>
       </c>
       <c r="K51" t="str">
-        <v>BHC Only</v>
+        <v>Mandatory</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Trading_Positions</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>BHCK2170</v>
+        <v>BHCK4340</v>
       </c>
       <c r="B52" t="str">
-        <v>BHC Total Assets</v>
+        <v>BHC Net Income</v>
       </c>
       <c r="C52" t="str">
         <v>FR Y-9C</v>
       </c>
       <c r="D52" t="str">
-        <v>HC-Line 12</v>
+        <v>HC-Line 14</v>
       </c>
       <c r="E52" t="str">
-        <v>BHC Balance Sheet</v>
+        <v>BHC Income</v>
       </c>
       <c r="F52" t="str">
-        <v>Consolidated total assets for bank holding company</v>
+        <v>Consolidated net income for bank holding company</v>
       </c>
       <c r="G52" t="str">
         <v>Thousands USD</v>
@@ -2210,7 +2363,7 @@
         <v>BHCK</v>
       </c>
       <c r="I52" t="str">
-        <v>2170</v>
+        <v>4340</v>
       </c>
       <c r="J52" t="str">
         <v>FR Y-9C</v>
@@ -2218,25 +2371,28 @@
       <c r="K52" t="str">
         <v>BHC Only</v>
       </c>
+      <c r="L52" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>BHCK3210</v>
+        <v>BHCK2170</v>
       </c>
       <c r="B53" t="str">
-        <v>BHC Total Equity</v>
+        <v>BHC Total Assets</v>
       </c>
       <c r="C53" t="str">
         <v>FR Y-9C</v>
       </c>
       <c r="D53" t="str">
-        <v>HC-Line 28</v>
+        <v>HC-Line 12</v>
       </c>
       <c r="E53" t="str">
         <v>BHC Balance Sheet</v>
       </c>
       <c r="F53" t="str">
-        <v>Total equity capital of bank holding company</v>
+        <v>Consolidated total assets for bank holding company</v>
       </c>
       <c r="G53" t="str">
         <v>Thousands USD</v>
@@ -2245,7 +2401,7 @@
         <v>BHCK</v>
       </c>
       <c r="I53" t="str">
-        <v>3210</v>
+        <v>2170</v>
       </c>
       <c r="J53" t="str">
         <v>FR Y-9C</v>
@@ -2253,25 +2409,28 @@
       <c r="K53" t="str">
         <v>BHC Only</v>
       </c>
+      <c r="L53" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>BHCKA223</v>
+        <v>BHCK3210</v>
       </c>
       <c r="B54" t="str">
-        <v>BHC CET1 Capital</v>
+        <v>BHC Total Equity</v>
       </c>
       <c r="C54" t="str">
         <v>FR Y-9C</v>
       </c>
       <c r="D54" t="str">
-        <v>HC-R Line 22</v>
+        <v>HC-Line 28</v>
       </c>
       <c r="E54" t="str">
-        <v>BHC Capital</v>
+        <v>BHC Balance Sheet</v>
       </c>
       <c r="F54" t="str">
-        <v>Common Equity Tier 1 capital for BHC</v>
+        <v>Total equity capital of bank holding company</v>
       </c>
       <c r="G54" t="str">
         <v>Thousands USD</v>
@@ -2280,18 +2439,59 @@
         <v>BHCK</v>
       </c>
       <c r="I54" t="str">
-        <v>A223</v>
+        <v>3210</v>
       </c>
       <c r="J54" t="str">
-        <v>Basel III</v>
+        <v>FR Y-9C</v>
       </c>
       <c r="K54" t="str">
         <v>BHC Only</v>
       </c>
+      <c r="L54" t="str">
+        <v>Risk_Metrics</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>BHCKA223</v>
+      </c>
+      <c r="B55" t="str">
+        <v>BHC CET1 Capital</v>
+      </c>
+      <c r="C55" t="str">
+        <v>FR Y-9C</v>
+      </c>
+      <c r="D55" t="str">
+        <v>HC-R Line 22</v>
+      </c>
+      <c r="E55" t="str">
+        <v>BHC Capital</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Common Equity Tier 1 capital for BHC</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Thousands USD</v>
+      </c>
+      <c r="H55" t="str">
+        <v>BHCK</v>
+      </c>
+      <c r="I55" t="str">
+        <v>A223</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Basel III</v>
+      </c>
+      <c r="K55" t="str">
+        <v>BHC Only</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Risk_Metrics</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L55"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>